<commit_message>
0226    console.stack bug修复 console.stack保存数据修改 await转译代码，bug修复 Tips，Setting升级为ts 入口文件 ts
</commit_message>
<xml_diff>
--- a/packages/模块进度.xlsx
+++ b/packages/模块进度.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\project\js\AnJsflScript-ts\packages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5E1EE3-49B0-46D8-9F0A-12B63B6E80D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816C11DD-E20D-48E1-8A6B-0BCAB4ABB37E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="25720" windowHeight="13800" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11682,40 +11682,44 @@
     <col min="5" max="5" width="8.6640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:3" ht="14.5">
+    <row r="4" spans="3:5" ht="14.5">
       <c r="C4" s="10" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="5" spans="3:3" ht="14.5">
+    <row r="5" spans="3:5" ht="14.5">
       <c r="C5" s="10" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="7" spans="3:3" ht="14.5">
+    <row r="7" spans="3:5" ht="14.5">
       <c r="C7" s="10" t="s">
         <v>492</v>
       </c>
-    </row>
-    <row r="8" spans="3:3">
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="3:5">
       <c r="C8" t="s">
         <v>493</v>
       </c>
-    </row>
-    <row r="9" spans="3:3" ht="14.5">
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="3:5" ht="14.5">
       <c r="C9" s="10" t="s">
         <v>494</v>
       </c>
-    </row>
-    <row r="10" spans="3:3">
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="3:5">
       <c r="C10" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="11" spans="3:3" ht="14.5">
+    <row r="11" spans="3:5" ht="14.5">
       <c r="C11" s="10" t="s">
         <v>496</v>
       </c>
+      <c r="E11" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>